<commit_message>
Clean project and add gitignore
</commit_message>
<xml_diff>
--- a/Data/Login_data.xlsx
+++ b/Data/Login_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\datn\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{11BA0CC2-D7DF-49F8-8684-2D6C54FDEDCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{485144D0-3FF8-45CA-8A1A-4021E11D91E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EB387E9C-8EEB-447F-B9EF-DC1E7398EA24}"/>
   </bookViews>
@@ -20,58 +20,91 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t xml:space="preserve">email,password,expected_result		</t>
-  </si>
-  <si>
-    <t xml:space="preserve">thuytien010524@gmail.com,Tien15,"Hi, Ph?m Tiên"		</t>
-  </si>
-  <si>
-    <t xml:space="preserve">,,Please fill out this field.		</t>
-  </si>
-  <si>
-    <t xml:space="preserve">,Tien15,Please fill out this field.		</t>
-  </si>
-  <si>
-    <t xml:space="preserve">thuytien010524@gmail.com,Ti,Thông tin ??ng nh?p không h?p l?.		</t>
-  </si>
-  <si>
-    <t>thuytien01gmail.com,Tien15,Please include an '@' in the email address. 'thuytien0	1g	mail.com' is missing an '@'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">thuytien010524@gmail.com,Tien13,Thông tin ??ng nh?p không h?p l?.		</t>
-  </si>
-  <si>
-    <t xml:space="preserve">thuytien01@gmail.com,Tien15,Thông tin ??ng nh?p không h?p l?.		</t>
-  </si>
-  <si>
-    <t>thuytien01@,Tien15,Please enter the correct code after the '@'. 'thuytien010524@'	i	s incomplete.</t>
-  </si>
-  <si>
-    <t>thuytien010524@@gmail.com,Tien15,A part following '@' should not contain the symb	ol	'@'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">thuytien010524@gmail..com,Tien15,'.' is used at a wrong position in 'gmail..com'.		</t>
-  </si>
-  <si>
-    <t xml:space="preserve">thuytien1524@gmail.com,,Please fill out this field.		</t>
-  </si>
-  <si>
-    <t xml:space="preserve">THUYTIEN010524@gmail.com,Tien15,"Hi, Ph?m Tiên"		</t>
-  </si>
-  <si>
-    <t xml:space="preserve">thuytien010524@gmail.com,Tien@123,"Hi, Ph?m Tiên"		</t>
-  </si>
-  <si>
-    <t xml:space="preserve">thuytien010524@gmail.com,TIEN150524,Thông tin ??ng nh?p không h?p l?		</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="26">
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t xml:space="preserve">expected_result	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">email	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thuytien010524@gmail.com		</t>
+  </si>
+  <si>
+    <t>Tien15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Please fill out this field.	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tien15	</t>
+  </si>
+  <si>
+    <t>Please fill out this field.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thuytien010524@gmail.com	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ti	</t>
+  </si>
+  <si>
+    <t>thuytien01gmail.com</t>
+  </si>
+  <si>
+    <t>Tien13</t>
+  </si>
+  <si>
+    <t>Thông tin đăng nhập không hợp lệ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thuytien01@gmail.com	</t>
+  </si>
+  <si>
+    <t>thuytien01@</t>
+  </si>
+  <si>
+    <t>thuytien010524@@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thuytien010524@gmail..com	</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thuytien1524@gmail.com	</t>
+  </si>
+  <si>
+    <t>'.' is used at a wrong position in 'gmail..com'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THUYTIEN010524@gmail.com		</t>
+  </si>
+  <si>
+    <t>TIEN150524</t>
+  </si>
+  <si>
+    <t>Hi, Phạm Tiên</t>
+  </si>
+  <si>
+    <t>Please include an '@' in the email address. 'thuytien01gmail.com' is missing an '@'.</t>
+  </si>
+  <si>
+    <t>Please enter a part following '@'. 'thuytien01@' is incomplete.</t>
+  </si>
+  <si>
+    <t>A part following '@' should not contain the symbol '@'.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,6 +235,14 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -504,7 +545,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -547,11 +588,14 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -585,6 +629,7 @@
     <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
     <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
     <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
@@ -925,85 +970,174 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E46DDEE-EE08-480E-B17F-BAE4FEFA5D63}">
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="29.88671875" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" customWidth="1"/>
+    <col min="3" max="3" width="71" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="B14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{C3AA9179-344C-400F-AAB1-F12D5667F9AF}"/>
+    <hyperlink ref="A5" r:id="rId2" xr:uid="{CB43E779-BE51-413C-AB33-DD94E891E0C8}"/>
+    <hyperlink ref="A7" r:id="rId3" xr:uid="{C760320F-CADD-4173-91DB-2B2E9531A2C2}"/>
+    <hyperlink ref="A8" r:id="rId4" xr:uid="{6CFDB494-39C3-4ACB-B34E-3339BF55A3FF}"/>
+    <hyperlink ref="A9" r:id="rId5" xr:uid="{B670E0A1-47D9-4B37-B240-7C0F1667D0F6}"/>
+    <hyperlink ref="A11" r:id="rId6" xr:uid="{F19489DE-66B0-4938-8878-8C8D490C4A0F}"/>
+    <hyperlink ref="A12" r:id="rId7" xr:uid="{4E56A7BA-F384-4C43-A2FA-BF00880A1745}"/>
+    <hyperlink ref="A13" r:id="rId8" xr:uid="{B3FDA717-1FB4-43F1-B694-0A27AA0C2EE7}"/>
+    <hyperlink ref="A14" r:id="rId9" xr:uid="{60237CDD-1082-4339-94D2-C100AB190B36}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>